<commit_message>
fullgame/FG-EMG-1: EMG1-FW-02 事件补洞新固件落表（FG19A N09～N16）
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#ChannelDecl-通道声明.xlsx
+++ b/Configs/GameConfig/Datas/fg/#ChannelDecl-通道声明.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N206"/>
+  <dimension ref="A1:N222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12406,6 +12406,934 @@
         <v>3</v>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="inlineStr"/>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>fw_scuttle.1</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>fw_scuttle</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>1</v>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>evt.death</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>1</v>
+      </c>
+      <c r="J207" t="n">
+        <v>0</v>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L207" t="n">
+        <v>0</v>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_scuttle.1</t>
+        </is>
+      </c>
+      <c r="N207" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr"/>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>fw_scuttle.2</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>fw_scuttle</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>2</v>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>grm.trig</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>spawn</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>4</v>
+      </c>
+      <c r="J208" t="n">
+        <v>0</v>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L208" t="n">
+        <v>0</v>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_scuttle.2</t>
+        </is>
+      </c>
+      <c r="N208" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr"/>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>fw_bouncefuse.1</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>fw_bouncefuse</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>1</v>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>evt.bounce</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>1</v>
+      </c>
+      <c r="J209" t="n">
+        <v>0</v>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>projectile;summon</t>
+        </is>
+      </c>
+      <c r="L209" t="n">
+        <v>0</v>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_bouncefuse.1</t>
+        </is>
+      </c>
+      <c r="N209" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr"/>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>fw_bouncefuse.2</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>fw_bouncefuse</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>2</v>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>grm.trig</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>spawn</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>1</v>
+      </c>
+      <c r="J210" t="n">
+        <v>0</v>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>projectile;summon</t>
+        </is>
+      </c>
+      <c r="L210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_bouncefuse.2</t>
+        </is>
+      </c>
+      <c r="N210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr"/>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>fw_piercefuse.1</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>fw_piercefuse</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>1</v>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>evt.pierce</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>1</v>
+      </c>
+      <c r="J211" t="n">
+        <v>0</v>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>projectile;melee;summon</t>
+        </is>
+      </c>
+      <c r="L211" t="n">
+        <v>0</v>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_piercefuse.1</t>
+        </is>
+      </c>
+      <c r="N211" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr"/>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>fw_piercefuse.2</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>fw_piercefuse</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>2</v>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>grm.trig</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>spawn</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>1</v>
+      </c>
+      <c r="J212" t="n">
+        <v>0</v>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>projectile;melee;summon</t>
+        </is>
+      </c>
+      <c r="L212" t="n">
+        <v>0</v>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_piercefuse.2</t>
+        </is>
+      </c>
+      <c r="N212" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr"/>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>fw_ventarc.1</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>fw_ventarc</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>1</v>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>evt.overheat</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>1</v>
+      </c>
+      <c r="J213" t="n">
+        <v>0</v>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L213" t="n">
+        <v>0</v>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_ventarc.1</t>
+        </is>
+      </c>
+      <c r="N213" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr"/>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>fw_ventarc.2</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>fw_ventarc</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>2</v>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>en.elec</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>inject</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>4</v>
+      </c>
+      <c r="J214" t="n">
+        <v>0</v>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L214" t="n">
+        <v>0</v>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_ventarc.2</t>
+        </is>
+      </c>
+      <c r="N214" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr"/>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>fw_coolback.1</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>fw_coolback</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>1</v>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>evt.cooled</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>1</v>
+      </c>
+      <c r="J215" t="n">
+        <v>0</v>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L215" t="n">
+        <v>0</v>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_coolback.1</t>
+        </is>
+      </c>
+      <c r="N215" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr"/>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>fw_coolback.2</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>fw_coolback</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>2</v>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>mat.coolant</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>emit</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>1</v>
+      </c>
+      <c r="J216" t="n">
+        <v>0</v>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L216" t="n">
+        <v>0</v>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_coolback.2</t>
+        </is>
+      </c>
+      <c r="N216" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr"/>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>fw_enterfuse.1</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>fw_enterfuse</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>1</v>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>evt.enter</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>1</v>
+      </c>
+      <c r="J217" t="n">
+        <v>0</v>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L217" t="n">
+        <v>0</v>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_enterfuse.1</t>
+        </is>
+      </c>
+      <c r="N217" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr"/>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>fw_enterfuse.2</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>fw_enterfuse</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>2</v>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>grm.trig</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>spawn</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>1</v>
+      </c>
+      <c r="J218" t="n">
+        <v>0</v>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L218" t="n">
+        <v>0</v>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_enterfuse.2</t>
+        </is>
+      </c>
+      <c r="N218" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr"/>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>fw_uplinkpulse.1</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>fw_uplinkpulse</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>1</v>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>evt.uplink</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>1</v>
+      </c>
+      <c r="J219" t="n">
+        <v>0</v>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L219" t="n">
+        <v>0</v>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_uplinkpulse.1</t>
+        </is>
+      </c>
+      <c r="N219" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr"/>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>fw_uplinkpulse.2</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>fw_uplinkpulse</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>2</v>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>fld.push</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>spawn</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>3</v>
+      </c>
+      <c r="J220" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L220" t="n">
+        <v>0</v>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_uplinkpulse.2</t>
+        </is>
+      </c>
+      <c r="N220" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr"/>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>fw_water.1</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>fw_water</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>1</v>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>evt.hit</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>1</v>
+      </c>
+      <c r="J221" t="n">
+        <v>0</v>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L221" t="n">
+        <v>0</v>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_water.1</t>
+        </is>
+      </c>
+      <c r="N221" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr"/>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>fw_water.2</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>fw_water</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>firmware</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>2</v>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>mat.water</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>emit</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>1</v>
+      </c>
+      <c r="J222" t="n">
+        <v>0</v>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="L222" t="n">
+        <v>0</v>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>emg.decl.fw_water.2</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>